<commit_message>
feat(tcs): Type tagging complete — Admin 100%, others 93-100%
Final coverage:
  Admin    617/618 TCs tagged  (Customers 2 deprecated TCs skipped)
  Buyer    553/571            (~97%)
  CP       278/292            (~95%)
  SM       243/247            (~98%)
  Total    1,691 / 1,728 explicit Type rows (~98%)

Remaining ~37 TCs are deprecated/legacy/sub-entries without standard
table block — auto-inference covers them in Excel via heuristic.

Each Excel module sheet now bifurcates by 11 type groups with banner
divider rows. Index sheet shows per-module type breakdown.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/manual-qa-repository/07-execution/TestCases-BuyerPortal.xlsx
+++ b/manual-qa-repository/07-execution/TestCases-BuyerPortal.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5970" uniqueCount="2826">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5972" uniqueCount="2828">
   <si>
     <t>CUSTOMER PORTAL — MASTER TEST CASE DOCUMENT</t>
   </si>
@@ -144,7 +144,7 @@
     <t>Work Progress</t>
   </si>
   <si>
-    <t>UI:17 · FUNC:10 · INT:10 · API:2 · NEG:8</t>
+    <t>UI:17 · FUNC:7 · BIZ:2 · INT:11 · API:1 · EDGE:4 · NEG:5</t>
   </si>
   <si>
     <t>Work Progress — 47 TCs</t>
@@ -8091,6 +8091,241 @@
     <t>Work Progress menu item visible regardless of allocation status</t>
   </si>
   <si>
+    <t>BYR_WRK_004</t>
+  </si>
+  <si>
+    <t>Page header / title rendered</t>
+  </si>
+  <si>
+    <t>Page open</t>
+  </si>
+  <si>
+    <t>1. Inspect H1 / header</t>
+  </si>
+  <si>
+    <t>Title clearly identifies "Work Progress" / "Construction Updates"</t>
+  </si>
+  <si>
+    <t>BYR_WRK_005</t>
+  </si>
+  <si>
+    <t>Work Progress — Content Rendering</t>
+  </si>
+  <si>
+    <t>Milestones listed with photos</t>
+  </si>
+  <si>
+    <t>CMS has at least one milestone published</t>
+  </si>
+  <si>
+    <t>Each milestone card shows photo, title and description</t>
+  </si>
+  <si>
+    <t>BYR_WRK_006</t>
+  </si>
+  <si>
+    <t>Milestone photos load without 404</t>
+  </si>
+  <si>
+    <t>1. Inspect network requests for image loads</t>
+  </si>
+  <si>
+    <t>All images return 200; no broken image icons</t>
+  </si>
+  <si>
+    <t>BYR_WRK_007</t>
+  </si>
+  <si>
+    <t>Milestone date label visible per card</t>
+  </si>
+  <si>
+    <t>1. Inspect milestone cards</t>
+  </si>
+  <si>
+    <t>Date label rendered (e.g., "March 2026") for each milestone</t>
+  </si>
+  <si>
+    <t>BYR_WRK_008</t>
+  </si>
+  <si>
+    <t>Stage description text rendered</t>
+  </si>
+  <si>
+    <t>1. Read description per card</t>
+  </si>
+  <si>
+    <t>Text describes the construction stage as configured in CMS</t>
+  </si>
+  <si>
+    <t>BYR_WRK_009</t>
+  </si>
+  <si>
+    <t>Milestones rendered in chronological order</t>
+  </si>
+  <si>
+    <t>Multiple milestones exist</t>
+  </si>
+  <si>
+    <t>1. Inspect date order of cards</t>
+  </si>
+  <si>
+    <t>Cards sorted (typically newest first or chronological per CMS config)</t>
+  </si>
+  <si>
+    <t>BYR_WRK_013</t>
+  </si>
+  <si>
+    <t>Work Progress — Read-Only Constraint</t>
+  </si>
+  <si>
+    <t>No comment / edit affordances rendered</t>
+  </si>
+  <si>
+    <t>1. Scan UI for input boxes, edit/delete icons</t>
+  </si>
+  <si>
+    <t>No editable controls; buyer cannot add content</t>
+  </si>
+  <si>
+    <t>BYR_WRK_020</t>
+  </si>
+  <si>
+    <t>Work Progress — Negative &amp; Edge Cases</t>
+  </si>
+  <si>
+    <t>Page responsive on mobile viewport</t>
+  </si>
+  <si>
+    <t>Resize to mobile (≤480px)</t>
+  </si>
+  <si>
+    <t>1. Inspect layout</t>
+  </si>
+  <si>
+    <t>Cards stack vertically; photos resize without overflow</t>
+  </si>
+  <si>
+    <t>BYR_WRK_021</t>
+  </si>
+  <si>
+    <t>Slow image load shows progressive placeholder</t>
+  </si>
+  <si>
+    <t>Throttle network to 3G</t>
+  </si>
+  <si>
+    <t>1. Reload page</t>
+  </si>
+  <si>
+    <t>Placeholder/skeleton shown while images load</t>
+  </si>
+  <si>
+    <t>BYR_WRK_025</t>
+  </si>
+  <si>
+    <t>Banner video autoplays muted+looped with no controls</t>
+  </si>
+  <si>
+    <t>`data.attributes.workBannerVideo.data.attributes.url` populated in Strapi</t>
+  </si>
+  <si>
+    <t>1. Inspect `&lt;video&gt;` element</t>
+  </si>
+  <si>
+    <t>Attributes: `muted, autoplay, loop, playsInline, preload="auto"`, NO `controls`. Buyer cannot pause/seek (KB-6, work-progress/page.js:37-48).</t>
+  </si>
+  <si>
+    <t>BYR_WRK_027</t>
+  </si>
+  <si>
+    <t>Swiper responsive breakpoints</t>
+  </si>
+  <si>
+    <t>Tower with ≥4 images</t>
+  </si>
+  <si>
+    <t>1. Resize viewport to 320 / 640 / 1024 / 1200 / 1600 px</t>
+  </si>
+  <si>
+    <t>slidesPerView = 1 / 2 / 3 / 4 / 4 respectively (TowerTabs.js:36-56).</t>
+  </si>
+  <si>
+    <t>BYR_WRK_030</t>
+  </si>
+  <si>
+    <t>No timestamp / "last updated" indicator</t>
+  </si>
+  <si>
+    <t>Tower carousel visible</t>
+  </si>
+  <si>
+    <t>1. Inspect page for last-updated text</t>
+  </si>
+  <si>
+    <t>None rendered (KB-8). Buyer cannot tell whether images are current. Document UX gap.</t>
+  </si>
+  <si>
+    <t>BYR_WRK_031</t>
+  </si>
+  <si>
+    <t>No upload/replace photo control rendered</t>
+  </si>
+  <si>
+    <t>Work Progress page open</t>
+  </si>
+  <si>
+    <t>1. Inspect DOM for `&lt;input type=file&gt;` or upload buttons</t>
+  </si>
+  <si>
+    <t>No upload affordances anywhere on page; consumption-only UI</t>
+  </si>
+  <si>
+    <t>BYR_WRK_032</t>
+  </si>
+  <si>
+    <t>No delete/remove control on any milestone card</t>
+  </si>
+  <si>
+    <t>Page with milestone cards</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Hover over each card
+2. Inspect for delete icon / kebab menu</t>
+  </si>
+  <si>
+    <t>No delete or kebab menu rendered; cards are display-only</t>
+  </si>
+  <si>
+    <t>BYR_WRK_035</t>
+  </si>
+  <si>
+    <t>Image right-click "save as" allowed (read-only consumption)</t>
+  </si>
+  <si>
+    <t>1. Right-click image → Save As</t>
+  </si>
+  <si>
+    <t>Standard browser save dialog appears; image downloadable per public asset (no DRM expected)</t>
+  </si>
+  <si>
+    <t>BYR_WRK_043</t>
+  </si>
+  <si>
+    <t>Tablet viewport (~768px) shows correct slidesPerView</t>
+  </si>
+  <si>
+    <t>Resize to ~768px width</t>
+  </si>
+  <si>
+    <t>1. Inspect carousel</t>
+  </si>
+  <si>
+    <t>slidesPerView = 3 (per breakpoint table BYR_WRK_027); no overflow, no overlap</t>
+  </si>
+  <si>
+    <t>━━━━━━━━━━  FUNCTIONAL TESTS  (7)  ━━━━━━━━━━</t>
+  </si>
+  <si>
     <t>BYR_WRK_002</t>
   </si>
   <si>
@@ -8104,99 +8339,6 @@
   </si>
   <si>
     <t>URL = `/work-progress`; page loads</t>
-  </si>
-  <si>
-    <t>BYR_WRK_003</t>
-  </si>
-  <si>
-    <t>Buyer in any journey state</t>
-  </si>
-  <si>
-    <t>1. Open `/work-progress` in pre-allocation and post-allocation states</t>
-  </si>
-  <si>
-    <t>Same content accessible in both states</t>
-  </si>
-  <si>
-    <t>BYR_WRK_004</t>
-  </si>
-  <si>
-    <t>Page header / title rendered</t>
-  </si>
-  <si>
-    <t>Page open</t>
-  </si>
-  <si>
-    <t>1. Inspect H1 / header</t>
-  </si>
-  <si>
-    <t>Title clearly identifies "Work Progress" / "Construction Updates"</t>
-  </si>
-  <si>
-    <t>BYR_WRK_005</t>
-  </si>
-  <si>
-    <t>Work Progress — Content Rendering</t>
-  </si>
-  <si>
-    <t>Milestones listed with photos</t>
-  </si>
-  <si>
-    <t>CMS has at least one milestone published</t>
-  </si>
-  <si>
-    <t>Each milestone card shows photo, title and description</t>
-  </si>
-  <si>
-    <t>BYR_WRK_006</t>
-  </si>
-  <si>
-    <t>Milestone photos load without 404</t>
-  </si>
-  <si>
-    <t>1. Inspect network requests for image loads</t>
-  </si>
-  <si>
-    <t>All images return 200; no broken image icons</t>
-  </si>
-  <si>
-    <t>BYR_WRK_007</t>
-  </si>
-  <si>
-    <t>Milestone date label visible per card</t>
-  </si>
-  <si>
-    <t>1. Inspect milestone cards</t>
-  </si>
-  <si>
-    <t>Date label rendered (e.g., "March 2026") for each milestone</t>
-  </si>
-  <si>
-    <t>BYR_WRK_008</t>
-  </si>
-  <si>
-    <t>Stage description text rendered</t>
-  </si>
-  <si>
-    <t>1. Read description per card</t>
-  </si>
-  <si>
-    <t>Text describes the construction stage as configured in CMS</t>
-  </si>
-  <si>
-    <t>BYR_WRK_009</t>
-  </si>
-  <si>
-    <t>Milestones rendered in chronological order</t>
-  </si>
-  <si>
-    <t>Multiple milestones exist</t>
-  </si>
-  <si>
-    <t>1. Inspect date order of cards</t>
-  </si>
-  <si>
-    <t>Cards sorted (typically newest first or chronological per CMS config)</t>
   </si>
   <si>
     <t>BYR_WRK_010</t>
@@ -8236,74 +8378,90 @@
 2. Reopen, click X</t>
   </si>
   <si>
-    <t>BYR_WRK_013</t>
-  </si>
-  <si>
-    <t>Work Progress — Read-Only Constraint</t>
-  </si>
-  <si>
-    <t>No comment / edit affordances rendered</t>
-  </si>
-  <si>
-    <t>1. Scan UI for input boxes, edit/delete icons</t>
-  </si>
-  <si>
-    <t>No editable controls; buyer cannot add content</t>
-  </si>
-  <si>
-    <t>BYR_WRK_031</t>
-  </si>
-  <si>
-    <t>No upload/replace photo control rendered</t>
-  </si>
-  <si>
-    <t>Work Progress page open</t>
-  </si>
-  <si>
-    <t>1. Inspect DOM for `&lt;input type=file&gt;` or upload buttons</t>
-  </si>
-  <si>
-    <t>No upload affordances anywhere on page; consumption-only UI</t>
-  </si>
-  <si>
-    <t>BYR_WRK_032</t>
-  </si>
-  <si>
-    <t>No delete/remove control on any milestone card</t>
-  </si>
-  <si>
-    <t>Page with milestone cards</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Hover over each card
-2. Inspect for delete icon / kebab menu</t>
-  </si>
-  <si>
-    <t>No delete or kebab menu rendered; cards are display-only</t>
-  </si>
-  <si>
-    <t>BYR_WRK_033</t>
-  </si>
-  <si>
-    <t>Right-click context menu does not expose admin actions</t>
-  </si>
-  <si>
-    <t>1. Right-click on milestone card and image</t>
-  </si>
-  <si>
-    <t>Only standard browser context menu; no custom admin/edit options leaked through</t>
-  </si>
-  <si>
-    <t>BYR_WRK_035</t>
-  </si>
-  <si>
-    <t>Image right-click "save as" allowed (read-only consumption)</t>
-  </si>
-  <si>
-    <t>1. Right-click image → Save As</t>
-  </si>
-  <si>
-    <t>Standard browser save dialog appears; image downloadable per public asset (no DRM expected)</t>
+    <t>BYR_WRK_028</t>
+  </si>
+  <si>
+    <t>Autoplay continues after manual swipe (disableOnInteraction=false)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Manually drag a slide
+2. Wait 3 seconds</t>
+  </si>
+  <si>
+    <t>Autoplay resumes at 2500ms delay (TowerTabs.js:31-34).</t>
+  </si>
+  <si>
+    <t>BYR_WRK_003</t>
+  </si>
+  <si>
+    <t>Buyer in any journey state</t>
+  </si>
+  <si>
+    <t>1. Open `/work-progress` in pre-allocation and post-allocation states</t>
+  </si>
+  <si>
+    <t>Same content accessible in both states</t>
+  </si>
+  <si>
+    <t>BYR_WRK_023</t>
+  </si>
+  <si>
+    <t>Per-buyer tower filter is dead code — buyer sees ALL towers</t>
+  </si>
+  <si>
+    <t>Buyer allocated to one tower (e.g., Crest)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open `/work-progress`
+2. Inspect tower tab list</t>
+  </si>
+  <si>
+    <t>ALL towers configured in Strapi shown, not just buyer's. Filter logic at TowerSection.js:14-31 is commented out (KB-2).</t>
+  </si>
+  <si>
+    <t>━━━━━━━━━━  INTEGRATION TESTS  (11)  ━━━━━━━━━━</t>
+  </si>
+  <si>
+    <t>BYR_WRK_015</t>
+  </si>
+  <si>
+    <t>Work Progress — CMS Sync &amp; Content Refresh</t>
+  </si>
+  <si>
+    <t>New milestone published in CMS appears on reload</t>
+  </si>
+  <si>
+    <t>Admin publishes new milestone in CMS</t>
+  </si>
+  <si>
+    <t>1. Reload `/work-progress`</t>
+  </si>
+  <si>
+    <t>New milestone card visible without code deploy</t>
+  </si>
+  <si>
+    <t>BYR_WRK_016</t>
+  </si>
+  <si>
+    <t>Removed milestone disappears on reload</t>
+  </si>
+  <si>
+    <t>Admin unpublishes a milestone</t>
+  </si>
+  <si>
+    <t>Card no longer rendered</t>
+  </si>
+  <si>
+    <t>BYR_WRK_017</t>
+  </si>
+  <si>
+    <t>Updated description reflected on reload</t>
+  </si>
+  <si>
+    <t>Admin edits milestone description</t>
+  </si>
+  <si>
+    <t>New text shown</t>
   </si>
   <si>
     <t>BYR_WRK_022</t>
@@ -8322,37 +8480,6 @@
     <t>URL = `&lt;strapi&gt;/api/projects/1?populate=deep` regardless of buyer's actual project (KB-1, urls.js:8). Document multi-project rollout BUG.</t>
   </si>
   <si>
-    <t>BYR_WRK_023</t>
-  </si>
-  <si>
-    <t>Per-buyer tower filter is dead code — buyer sees ALL towers</t>
-  </si>
-  <si>
-    <t>Buyer allocated to one tower (e.g., Crest)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open `/work-progress`
-2. Inspect tower tab list</t>
-  </si>
-  <si>
-    <t>ALL towers configured in Strapi shown, not just buyer's. Filter logic at TowerSection.js:14-31 is commented out (KB-2).</t>
-  </si>
-  <si>
-    <t>BYR_WRK_025</t>
-  </si>
-  <si>
-    <t>Banner video autoplays muted+looped with no controls</t>
-  </si>
-  <si>
-    <t>`data.attributes.workBannerVideo.data.attributes.url` populated in Strapi</t>
-  </si>
-  <si>
-    <t>1. Inspect `&lt;video&gt;` element</t>
-  </si>
-  <si>
-    <t>Attributes: `muted, autoplay, loop, playsInline, preload="auto"`, NO `controls`. Buyer cannot pause/seek (KB-6, work-progress/page.js:37-48).</t>
-  </si>
-  <si>
     <t>BYR_WRK_026</t>
   </si>
   <si>
@@ -8366,37 +8493,6 @@
   </si>
   <si>
     <t>H2 = `.title`, P = `.subtitle` from that entry. If absent: H2 and P render empty without showing "undefined" (work-progress/page.js:17-19, 25-26).</t>
-  </si>
-  <si>
-    <t>BYR_WRK_027</t>
-  </si>
-  <si>
-    <t>Swiper responsive breakpoints</t>
-  </si>
-  <si>
-    <t>Tower with ≥4 images</t>
-  </si>
-  <si>
-    <t>1. Resize viewport to 320 / 640 / 1024 / 1200 / 1600 px</t>
-  </si>
-  <si>
-    <t>slidesPerView = 1 / 2 / 3 / 4 / 4 respectively (TowerTabs.js:36-56).</t>
-  </si>
-  <si>
-    <t>BYR_WRK_028</t>
-  </si>
-  <si>
-    <t>Autoplay continues after manual swipe (disableOnInteraction=false)</t>
-  </si>
-  <si>
-    <t>Tower carousel visible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Manually drag a slide
-2. Wait 3 seconds</t>
-  </si>
-  <si>
-    <t>Autoplay resumes at 2500ms delay (TowerTabs.js:31-34).</t>
   </si>
   <si>
     <t>BYR_WRK_029</t>
@@ -8416,93 +8512,6 @@
     <t>NO buyer notification on any channel. No mailer, push, WebSocket, or in-app badge for work-progress events (KB-9, FSD §5). Buyer must visit page to see updates. Document as missing-feature.</t>
   </si>
   <si>
-    <t>BYR_WRK_030</t>
-  </si>
-  <si>
-    <t>No timestamp / "last updated" indicator</t>
-  </si>
-  <si>
-    <t>1. Inspect page for last-updated text</t>
-  </si>
-  <si>
-    <t>None rendered (KB-8). Buyer cannot tell whether images are current. Document UX gap.</t>
-  </si>
-  <si>
-    <t>BYR_WRK_015</t>
-  </si>
-  <si>
-    <t>Work Progress — CMS Sync &amp; Content Refresh</t>
-  </si>
-  <si>
-    <t>New milestone published in CMS appears on reload</t>
-  </si>
-  <si>
-    <t>Admin publishes new milestone in CMS</t>
-  </si>
-  <si>
-    <t>1. Reload `/work-progress`</t>
-  </si>
-  <si>
-    <t>New milestone card visible without code deploy</t>
-  </si>
-  <si>
-    <t>BYR_WRK_016</t>
-  </si>
-  <si>
-    <t>Removed milestone disappears on reload</t>
-  </si>
-  <si>
-    <t>Admin unpublishes a milestone</t>
-  </si>
-  <si>
-    <t>1. Reload page</t>
-  </si>
-  <si>
-    <t>Card no longer rendered</t>
-  </si>
-  <si>
-    <t>BYR_WRK_017</t>
-  </si>
-  <si>
-    <t>Updated description reflected on reload</t>
-  </si>
-  <si>
-    <t>Admin edits milestone description</t>
-  </si>
-  <si>
-    <t>New text shown</t>
-  </si>
-  <si>
-    <t>BYR_WRK_024</t>
-  </si>
-  <si>
-    <t>Strapi outage leaves "Loading tower data..." placeholder forever</t>
-  </si>
-  <si>
-    <t>Block Strapi URL in network</t>
-  </si>
-  <si>
-    <t>1. Open `/work-progress`</t>
-  </si>
-  <si>
-    <t>Banner section renders (or doesn't, depending on cache). Tower section shows "Loading tower data..." indefinitely; error state is commented out (KB-5, TowerSection.js:11).</t>
-  </si>
-  <si>
-    <t>BYR_WRK_034</t>
-  </si>
-  <si>
-    <t>Attempted PUT to Strapi from buyer rejected</t>
-  </si>
-  <si>
-    <t>Buyer JWT in hand</t>
-  </si>
-  <si>
-    <t>1. `PUT &lt;strapi&gt;/api/projects/1` with buyer auth header</t>
-  </si>
-  <si>
-    <t>Rejected — Strapi requires admin auth; buyer JWT not accepted for writes (verify CORS/auth boundary)</t>
-  </si>
-  <si>
     <t>BYR_WRK_037</t>
   </si>
   <si>
@@ -8578,7 +8587,7 @@
     <t>New video URL active; muted+autoplay+loop attributes preserved (BYR_WRK_025)</t>
   </si>
   <si>
-    <t>━━━━━━━━━━  API TESTS  (2)  ━━━━━━━━━━</t>
+    <t>━━━━━━━━━━  API TESTS  (1)  ━━━━━━━━━━</t>
   </si>
   <si>
     <t>BYR_WRK_014</t>
@@ -8596,27 +8605,9 @@
     <t>404 or 403 — no buyer-write endpoint exists</t>
   </si>
   <si>
-    <t>BYR_WRK_036</t>
-  </si>
-  <si>
-    <t>Buyer cannot inject milestone via direct API call</t>
-  </si>
-  <si>
-    <t>Buyer token</t>
-  </si>
-  <si>
-    <t>1. `POST /api/v1/user/work-progress` or any guessed XR backend route</t>
-  </si>
-  <si>
-    <t>404 — no such route exists (FSD §6); confirms no buyer write surface</t>
-  </si>
-  <si>
     <t>BYR_WRK_018</t>
   </si>
   <si>
-    <t>Work Progress — Negative &amp; Edge Cases</t>
-  </si>
-  <si>
     <t>Empty state when no milestones published</t>
   </si>
   <si>
@@ -8627,45 +8618,6 @@
   </si>
   <si>
     <t>Empty state ("No updates yet") shown; no broken layout</t>
-  </si>
-  <si>
-    <t>BYR_WRK_019</t>
-  </si>
-  <si>
-    <t>CMS outage shows graceful fallback</t>
-  </si>
-  <si>
-    <t>CMS API simulated down</t>
-  </si>
-  <si>
-    <t>Friendly error or cached content; no app crash</t>
-  </si>
-  <si>
-    <t>BYR_WRK_020</t>
-  </si>
-  <si>
-    <t>Page responsive on mobile viewport</t>
-  </si>
-  <si>
-    <t>Resize to mobile (≤480px)</t>
-  </si>
-  <si>
-    <t>1. Inspect layout</t>
-  </si>
-  <si>
-    <t>Cards stack vertically; photos resize without overflow</t>
-  </si>
-  <si>
-    <t>BYR_WRK_021</t>
-  </si>
-  <si>
-    <t>Slow image load shows progressive placeholder</t>
-  </si>
-  <si>
-    <t>Throttle network to 3G</t>
-  </si>
-  <si>
-    <t>Placeholder/skeleton shown while images load</t>
   </si>
   <si>
     <t>BYR_WRK_042</t>
@@ -8684,21 +8636,6 @@
     <t>Broken image slot shows placeholder; remaining slides render normally; Swiper not blocked</t>
   </si>
   <si>
-    <t>BYR_WRK_043</t>
-  </si>
-  <si>
-    <t>Tablet viewport (~768px) shows correct slidesPerView</t>
-  </si>
-  <si>
-    <t>Resize to ~768px width</t>
-  </si>
-  <si>
-    <t>1. Inspect carousel</t>
-  </si>
-  <si>
-    <t>slidesPerView = 3 (per breakpoint table BYR_WRK_027); no overflow, no overlap</t>
-  </si>
-  <si>
     <t>BYR_WRK_044</t>
   </si>
   <si>
@@ -8724,6 +8661,75 @@
   </si>
   <si>
     <t>TowerSection silently absent (no "No updates yet" message per BYR_WRK_018 / KB-4); rest of page (banner, header) renders without crash</t>
+  </si>
+  <si>
+    <t>BYR_WRK_019</t>
+  </si>
+  <si>
+    <t>CMS outage shows graceful fallback</t>
+  </si>
+  <si>
+    <t>CMS API simulated down</t>
+  </si>
+  <si>
+    <t>Friendly error or cached content; no app crash</t>
+  </si>
+  <si>
+    <t>BYR_WRK_024</t>
+  </si>
+  <si>
+    <t>Strapi outage leaves "Loading tower data..." placeholder forever</t>
+  </si>
+  <si>
+    <t>Block Strapi URL in network</t>
+  </si>
+  <si>
+    <t>1. Open `/work-progress`</t>
+  </si>
+  <si>
+    <t>Banner section renders (or doesn't, depending on cache). Tower section shows "Loading tower data..." indefinitely; error state is commented out (KB-5, TowerSection.js:11).</t>
+  </si>
+  <si>
+    <t>BYR_WRK_033</t>
+  </si>
+  <si>
+    <t>Right-click context menu does not expose admin actions</t>
+  </si>
+  <si>
+    <t>1. Right-click on milestone card and image</t>
+  </si>
+  <si>
+    <t>Only standard browser context menu; no custom admin/edit options leaked through</t>
+  </si>
+  <si>
+    <t>BYR_WRK_034</t>
+  </si>
+  <si>
+    <t>Attempted PUT to Strapi from buyer rejected</t>
+  </si>
+  <si>
+    <t>Buyer JWT in hand</t>
+  </si>
+  <si>
+    <t>1. `PUT &lt;strapi&gt;/api/projects/1` with buyer auth header</t>
+  </si>
+  <si>
+    <t>Rejected — Strapi requires admin auth; buyer JWT not accepted for writes (verify CORS/auth boundary)</t>
+  </si>
+  <si>
+    <t>BYR_WRK_036</t>
+  </si>
+  <si>
+    <t>Buyer cannot inject milestone via direct API call</t>
+  </si>
+  <si>
+    <t>Buyer token</t>
+  </si>
+  <si>
+    <t>1. `POST /api/v1/user/work-progress` or any guessed XR backend route</t>
+  </si>
+  <si>
+    <t>404 — no such route exists (FSD §6); confirms no buyer write surface</t>
   </si>
 </sst>
 </file>
@@ -13215,7 +13221,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -13323,154 +13329,154 @@
       </c>
     </row>
     <row r="5" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="18" t="s">
         <v>2618</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="19" t="s">
         <v>2614</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="19" t="s">
         <v>2619</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="19" t="s">
         <v>2620</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="19" t="s">
         <v>2621</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="G5" s="19" t="s">
         <v>2622</v>
       </c>
-      <c r="H5" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="I5" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="J5" s="13" t="s">
+      <c r="H5" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="I5" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="J5" s="19" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>2623</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>2624</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>2625</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>2626</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>933</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>2627</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="I6" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="J6" s="13" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="6" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="18" t="s">
-        <v>2623</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>2614</v>
-      </c>
-      <c r="C6" s="20" t="s">
+    <row r="7" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="15" t="s">
+        <v>2628</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>2624</v>
+      </c>
+      <c r="C7" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="D6" s="19" t="s">
-        <v>1266</v>
-      </c>
-      <c r="E6" s="19" t="s">
+      <c r="D7" s="16" t="s">
+        <v>2629</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>2620</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>2630</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>2631</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="I7" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="J7" s="16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="15" t="s">
+        <v>2632</v>
+      </c>
+      <c r="B8" s="16" t="s">
         <v>2624</v>
       </c>
-      <c r="F6" s="19" t="s">
-        <v>2625</v>
-      </c>
-      <c r="G6" s="19" t="s">
-        <v>2626</v>
-      </c>
-      <c r="H6" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="I6" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="J6" s="19" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="18" t="s">
-        <v>2627</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>2614</v>
-      </c>
-      <c r="C7" s="20" t="s">
+      <c r="C8" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="D7" s="19" t="s">
-        <v>2628</v>
-      </c>
-      <c r="E7" s="19" t="s">
-        <v>2629</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>2630</v>
-      </c>
-      <c r="G7" s="19" t="s">
-        <v>2631</v>
-      </c>
-      <c r="H7" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="I7" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="J7" s="19" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="8" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
-        <v>2632</v>
-      </c>
-      <c r="B8" s="13" t="s">
+      <c r="D8" s="16" t="s">
         <v>2633</v>
       </c>
-      <c r="C8" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="D8" s="13" t="s">
+      <c r="E8" s="16" t="s">
+        <v>2620</v>
+      </c>
+      <c r="F8" s="16" t="s">
         <v>2634</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="G8" s="16" t="s">
         <v>2635</v>
       </c>
-      <c r="F8" s="13" t="s">
-        <v>933</v>
-      </c>
-      <c r="G8" s="13" t="s">
-        <v>2636</v>
-      </c>
-      <c r="H8" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="I8" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="J8" s="13" t="s">
-        <v>63</v>
+      <c r="H8" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="I8" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="J8" s="16" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="9" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
-        <v>2637</v>
+        <v>2636</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>2633</v>
+        <v>2624</v>
       </c>
       <c r="C9" s="17" t="s">
         <v>58</v>
       </c>
       <c r="D9" s="16" t="s">
+        <v>2637</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>2620</v>
+      </c>
+      <c r="F9" s="16" t="s">
         <v>2638</v>
       </c>
-      <c r="E9" s="16" t="s">
-        <v>2629</v>
-      </c>
-      <c r="F9" s="16" t="s">
+      <c r="G9" s="16" t="s">
         <v>2639</v>
-      </c>
-      <c r="G9" s="16" t="s">
-        <v>2640</v>
       </c>
       <c r="H9" s="16" t="s">
         <v>42</v>
@@ -13483,35 +13489,35 @@
       </c>
     </row>
     <row r="10" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="18" t="s">
+        <v>2640</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>2624</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="D10" s="19" t="s">
         <v>2641</v>
       </c>
-      <c r="B10" s="16" t="s">
-        <v>2633</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" s="16" t="s">
+      <c r="E10" s="19" t="s">
         <v>2642</v>
       </c>
-      <c r="E10" s="16" t="s">
-        <v>2629</v>
-      </c>
-      <c r="F10" s="16" t="s">
+      <c r="F10" s="19" t="s">
         <v>2643</v>
       </c>
-      <c r="G10" s="16" t="s">
+      <c r="G10" s="19" t="s">
         <v>2644</v>
       </c>
-      <c r="H10" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="I10" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="J10" s="16" t="s">
-        <v>10</v>
+      <c r="H10" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="I10" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="J10" s="19" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="11" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -13519,22 +13525,22 @@
         <v>2645</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>2633</v>
+        <v>2646</v>
       </c>
       <c r="C11" s="17" t="s">
         <v>58</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>2646</v>
+        <v>2647</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>2629</v>
+        <v>2620</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>2647</v>
+        <v>2648</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>2648</v>
+        <v>2649</v>
       </c>
       <c r="H11" s="16" t="s">
         <v>42</v>
@@ -13548,25 +13554,25 @@
     </row>
     <row r="12" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
-        <v>2649</v>
+        <v>2650</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>2633</v>
+        <v>2651</v>
       </c>
       <c r="C12" s="20" t="s">
         <v>58</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>2650</v>
+        <v>2652</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>2651</v>
+        <v>2653</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>2652</v>
+        <v>2654</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="H12" s="19" t="s">
         <v>42</v>
@@ -13580,25 +13586,25 @@
     </row>
     <row r="13" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="18" t="s">
-        <v>2654</v>
+        <v>2656</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>2633</v>
+        <v>2651</v>
       </c>
       <c r="C13" s="20" t="s">
         <v>58</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>2655</v>
+        <v>2657</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>2656</v>
+        <v>2658</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>2657</v>
+        <v>2659</v>
       </c>
       <c r="G13" s="19" t="s">
-        <v>2658</v>
+        <v>2660</v>
       </c>
       <c r="H13" s="19" t="s">
         <v>42</v>
@@ -13607,30 +13613,30 @@
         <v>42</v>
       </c>
       <c r="J13" s="19" t="s">
-        <v>79</v>
+        <v>328</v>
       </c>
     </row>
     <row r="14" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
-        <v>2659</v>
+        <v>2661</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>2633</v>
+        <v>146</v>
       </c>
       <c r="C14" s="20" t="s">
         <v>58</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>2660</v>
+        <v>2662</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>2661</v>
+        <v>2663</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>2662</v>
+        <v>2664</v>
       </c>
       <c r="G14" s="19" t="s">
-        <v>2663</v>
+        <v>2665</v>
       </c>
       <c r="H14" s="19" t="s">
         <v>42</v>
@@ -13639,30 +13645,30 @@
         <v>42</v>
       </c>
       <c r="J14" s="19" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="15" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
-        <v>2664</v>
+        <v>2666</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>2633</v>
+        <v>146</v>
       </c>
       <c r="C15" s="20" t="s">
         <v>58</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>1219</v>
+        <v>2667</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>1215</v>
+        <v>2668</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>2665</v>
+        <v>2669</v>
       </c>
       <c r="G15" s="19" t="s">
-        <v>1221</v>
+        <v>2670</v>
       </c>
       <c r="H15" s="19" t="s">
         <v>42</v>
@@ -13675,58 +13681,58 @@
       </c>
     </row>
     <row r="16" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="15" t="s">
-        <v>2666</v>
-      </c>
-      <c r="B16" s="16" t="s">
-        <v>2667</v>
-      </c>
-      <c r="C16" s="17" t="s">
+      <c r="A16" s="18" t="s">
+        <v>2671</v>
+      </c>
+      <c r="B16" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="C16" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="D16" s="16" t="s">
-        <v>2668</v>
-      </c>
-      <c r="E16" s="16" t="s">
-        <v>2629</v>
-      </c>
-      <c r="F16" s="16" t="s">
-        <v>2669</v>
-      </c>
-      <c r="G16" s="16" t="s">
-        <v>2670</v>
-      </c>
-      <c r="H16" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="I16" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="J16" s="16" t="s">
-        <v>10</v>
+      <c r="D16" s="19" t="s">
+        <v>2672</v>
+      </c>
+      <c r="E16" s="19" t="s">
+        <v>2673</v>
+      </c>
+      <c r="F16" s="19" t="s">
+        <v>2674</v>
+      </c>
+      <c r="G16" s="19" t="s">
+        <v>2675</v>
+      </c>
+      <c r="H16" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="I16" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="J16" s="19" t="s">
+        <v>328</v>
       </c>
     </row>
     <row r="17" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>2671</v>
+        <v>2676</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>2667</v>
+        <v>2646</v>
       </c>
       <c r="C17" s="17" t="s">
         <v>58</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>2672</v>
+        <v>2677</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>2673</v>
+        <v>2678</v>
       </c>
       <c r="F17" s="16" t="s">
-        <v>2674</v>
+        <v>2679</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>2675</v>
+        <v>2680</v>
       </c>
       <c r="H17" s="16" t="s">
         <v>42</v>
@@ -13740,25 +13746,25 @@
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>2676</v>
+        <v>2681</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>2667</v>
+        <v>2646</v>
       </c>
       <c r="C18" s="17" t="s">
         <v>58</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>2677</v>
+        <v>2682</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>2678</v>
+        <v>2683</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>2679</v>
+        <v>2684</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>2680</v>
+        <v>2685</v>
       </c>
       <c r="H18" s="16" t="s">
         <v>42</v>
@@ -13772,25 +13778,25 @@
     </row>
     <row r="19" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
-        <v>2681</v>
+        <v>2686</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>2667</v>
+        <v>2646</v>
       </c>
       <c r="C19" s="20" t="s">
         <v>58</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>2682</v>
+        <v>2687</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>2629</v>
+        <v>2620</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>2683</v>
+        <v>2688</v>
       </c>
       <c r="G19" s="19" t="s">
-        <v>2684</v>
+        <v>2689</v>
       </c>
       <c r="H19" s="19" t="s">
         <v>42</v>
@@ -13804,25 +13810,25 @@
     </row>
     <row r="20" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="18" t="s">
-        <v>2685</v>
+        <v>2690</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>2667</v>
+        <v>2651</v>
       </c>
       <c r="C20" s="20" t="s">
         <v>58</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>2686</v>
+        <v>2691</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>2629</v>
+        <v>2692</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>2687</v>
+        <v>2693</v>
       </c>
       <c r="G20" s="19" t="s">
-        <v>2688</v>
+        <v>2694</v>
       </c>
       <c r="H20" s="19" t="s">
         <v>42</v>
@@ -13836,7 +13842,7 @@
     </row>
     <row r="21" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>399</v>
+        <v>2695</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
@@ -13848,59 +13854,59 @@
       <c r="I21" s="11"/>
       <c r="J21" s="11"/>
     </row>
-    <row r="22" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="15" t="s">
-        <v>2689</v>
-      </c>
-      <c r="B22" s="16" t="s">
+    <row r="22" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>2696</v>
+      </c>
+      <c r="B22" s="13" t="s">
         <v>2614</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="C22" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="D22" s="16" t="s">
-        <v>2690</v>
-      </c>
-      <c r="E22" s="16" t="s">
-        <v>2691</v>
-      </c>
-      <c r="F22" s="16" t="s">
-        <v>2692</v>
-      </c>
-      <c r="G22" s="16" t="s">
-        <v>2693</v>
-      </c>
-      <c r="H22" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="I22" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="J22" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="23" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D22" s="13" t="s">
+        <v>2697</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>2698</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>2699</v>
+      </c>
+      <c r="G22" s="13" t="s">
+        <v>2700</v>
+      </c>
+      <c r="H22" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="I22" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="J22" s="13" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
-        <v>2694</v>
+        <v>2701</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>2614</v>
+        <v>2624</v>
       </c>
       <c r="C23" s="20" t="s">
         <v>94</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>2695</v>
+        <v>2702</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>2696</v>
+        <v>2703</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>2697</v>
+        <v>2704</v>
       </c>
       <c r="G23" s="19" t="s">
-        <v>2698</v>
+        <v>2705</v>
       </c>
       <c r="H23" s="19" t="s">
         <v>42</v>
@@ -13914,25 +13920,25 @@
     </row>
     <row r="24" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="18" t="s">
-        <v>2699</v>
+        <v>2706</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>146</v>
+        <v>2624</v>
       </c>
       <c r="C24" s="20" t="s">
         <v>94</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>2700</v>
+        <v>2707</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>2701</v>
+        <v>2708</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>2702</v>
+        <v>2709</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>2703</v>
+        <v>2710</v>
       </c>
       <c r="H24" s="19" t="s">
         <v>42</v>
@@ -13941,30 +13947,30 @@
         <v>42</v>
       </c>
       <c r="J24" s="19" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="25" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="25" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>2704</v>
+        <v>2711</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>2614</v>
+        <v>2624</v>
       </c>
       <c r="C25" s="20" t="s">
         <v>94</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>2705</v>
+        <v>1219</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>2706</v>
+        <v>1215</v>
       </c>
       <c r="F25" s="19" t="s">
-        <v>2707</v>
+        <v>2712</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>2708</v>
+        <v>1221</v>
       </c>
       <c r="H25" s="19" t="s">
         <v>42</v>
@@ -13973,12 +13979,12 @@
         <v>42</v>
       </c>
       <c r="J25" s="19" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="26" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="26" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="18" t="s">
-        <v>2709</v>
+        <v>2713</v>
       </c>
       <c r="B26" s="19" t="s">
         <v>146</v>
@@ -13987,16 +13993,16 @@
         <v>94</v>
       </c>
       <c r="D26" s="19" t="s">
-        <v>2710</v>
+        <v>2714</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>2711</v>
+        <v>2673</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>2712</v>
+        <v>2715</v>
       </c>
       <c r="G26" s="19" t="s">
-        <v>2713</v>
+        <v>2716</v>
       </c>
       <c r="H26" s="19" t="s">
         <v>42</v>
@@ -14008,9 +14014,9 @@
         <v>328</v>
       </c>
     </row>
-    <row r="27" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="18" t="s">
-        <v>2714</v>
+        <v>145</v>
       </c>
       <c r="B27" s="19" t="s">
         <v>146</v>
@@ -14019,16 +14025,16 @@
         <v>94</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>2715</v>
+        <v>147</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>2716</v>
+        <v>42</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>2717</v>
+        <v>42</v>
       </c>
       <c r="G27" s="19" t="s">
-        <v>2718</v>
+        <v>42</v>
       </c>
       <c r="H27" s="19" t="s">
         <v>42</v>
@@ -14037,12 +14043,12 @@
         <v>42</v>
       </c>
       <c r="J27" s="19" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="28" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="28" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="18" t="s">
-        <v>2719</v>
+        <v>148</v>
       </c>
       <c r="B28" s="19" t="s">
         <v>146</v>
@@ -14051,16 +14057,16 @@
         <v>94</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>2720</v>
+        <v>149</v>
       </c>
       <c r="E28" s="19" t="s">
-        <v>2721</v>
+        <v>42</v>
       </c>
       <c r="F28" s="19" t="s">
-        <v>2722</v>
+        <v>42</v>
       </c>
       <c r="G28" s="19" t="s">
-        <v>2723</v>
+        <v>42</v>
       </c>
       <c r="H28" s="19" t="s">
         <v>42</v>
@@ -14069,62 +14075,44 @@
         <v>42</v>
       </c>
       <c r="J28" s="19" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="29" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="18" t="s">
-        <v>2724</v>
-      </c>
-      <c r="B29" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="C29" s="20" t="s">
-        <v>94</v>
-      </c>
-      <c r="D29" s="19" t="s">
-        <v>2725</v>
-      </c>
-      <c r="E29" s="19" t="s">
-        <v>2716</v>
-      </c>
-      <c r="F29" s="19" t="s">
-        <v>2726</v>
-      </c>
-      <c r="G29" s="19" t="s">
-        <v>2727</v>
-      </c>
-      <c r="H29" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="I29" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="J29" s="19" t="s">
-        <v>328</v>
-      </c>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
+        <v>2528</v>
+      </c>
+      <c r="B29" s="11"/>
+      <c r="C29" s="11"/>
+      <c r="D29" s="11"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="11"/>
+      <c r="G29" s="11"/>
+      <c r="H29" s="11"/>
+      <c r="I29" s="11"/>
+      <c r="J29" s="11"/>
     </row>
     <row r="30" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="18" t="s">
-        <v>145</v>
+        <v>2717</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>146</v>
+        <v>2614</v>
       </c>
       <c r="C30" s="20" t="s">
-        <v>94</v>
+        <v>183</v>
       </c>
       <c r="D30" s="19" t="s">
-        <v>147</v>
+        <v>1266</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>42</v>
+        <v>2718</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>42</v>
+        <v>2719</v>
       </c>
       <c r="G30" s="19" t="s">
-        <v>42</v>
+        <v>2720</v>
       </c>
       <c r="H30" s="19" t="s">
         <v>42</v>
@@ -14133,30 +14121,30 @@
         <v>42</v>
       </c>
       <c r="J30" s="19" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="31" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="31" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="18" t="s">
-        <v>148</v>
+        <v>2721</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>146</v>
+        <v>2614</v>
       </c>
       <c r="C31" s="20" t="s">
-        <v>94</v>
+        <v>183</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>149</v>
+        <v>2722</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>42</v>
+        <v>2723</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>42</v>
+        <v>2724</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>42</v>
+        <v>2725</v>
       </c>
       <c r="H31" s="19" t="s">
         <v>42</v>
@@ -14165,12 +14153,12 @@
         <v>42</v>
       </c>
       <c r="J31" s="19" t="s">
-        <v>42</v>
+        <v>79</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
-        <v>2042</v>
+        <v>2726</v>
       </c>
       <c r="B32" s="11"/>
       <c r="C32" s="11"/>
@@ -14184,25 +14172,25 @@
     </row>
     <row r="33" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
+        <v>2727</v>
+      </c>
+      <c r="B33" s="16" t="s">
         <v>2728</v>
-      </c>
-      <c r="B33" s="16" t="s">
-        <v>2729</v>
       </c>
       <c r="C33" s="17" t="s">
         <v>205</v>
       </c>
       <c r="D33" s="16" t="s">
+        <v>2729</v>
+      </c>
+      <c r="E33" s="16" t="s">
         <v>2730</v>
       </c>
-      <c r="E33" s="16" t="s">
+      <c r="F33" s="16" t="s">
         <v>2731</v>
       </c>
-      <c r="F33" s="16" t="s">
+      <c r="G33" s="16" t="s">
         <v>2732</v>
-      </c>
-      <c r="G33" s="16" t="s">
-        <v>2733</v>
       </c>
       <c r="H33" s="16" t="s">
         <v>42</v>
@@ -14216,25 +14204,25 @@
     </row>
     <row r="34" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="18" t="s">
-        <v>2734</v>
+        <v>2733</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>2729</v>
+        <v>2728</v>
       </c>
       <c r="C34" s="20" t="s">
         <v>205</v>
       </c>
       <c r="D34" s="19" t="s">
+        <v>2734</v>
+      </c>
+      <c r="E34" s="19" t="s">
         <v>2735</v>
       </c>
-      <c r="E34" s="19" t="s">
+      <c r="F34" s="19" t="s">
+        <v>2659</v>
+      </c>
+      <c r="G34" s="19" t="s">
         <v>2736</v>
-      </c>
-      <c r="F34" s="19" t="s">
-        <v>2737</v>
-      </c>
-      <c r="G34" s="19" t="s">
-        <v>2738</v>
       </c>
       <c r="H34" s="19" t="s">
         <v>42</v>
@@ -14248,25 +14236,25 @@
     </row>
     <row r="35" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="18" t="s">
-        <v>2739</v>
+        <v>2737</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>2729</v>
+        <v>2728</v>
       </c>
       <c r="C35" s="20" t="s">
         <v>205</v>
       </c>
       <c r="D35" s="19" t="s">
+        <v>2738</v>
+      </c>
+      <c r="E35" s="19" t="s">
+        <v>2739</v>
+      </c>
+      <c r="F35" s="19" t="s">
+        <v>2659</v>
+      </c>
+      <c r="G35" s="19" t="s">
         <v>2740</v>
-      </c>
-      <c r="E35" s="19" t="s">
-        <v>2741</v>
-      </c>
-      <c r="F35" s="19" t="s">
-        <v>2737</v>
-      </c>
-      <c r="G35" s="19" t="s">
-        <v>2742</v>
       </c>
       <c r="H35" s="19" t="s">
         <v>42</v>
@@ -14278,91 +14266,91 @@
         <v>79</v>
       </c>
     </row>
-    <row r="36" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="18" t="s">
+    <row r="36" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="15" t="s">
+        <v>2741</v>
+      </c>
+      <c r="B36" s="16" t="s">
+        <v>2614</v>
+      </c>
+      <c r="C36" s="17" t="s">
+        <v>205</v>
+      </c>
+      <c r="D36" s="16" t="s">
+        <v>2742</v>
+      </c>
+      <c r="E36" s="16" t="s">
         <v>2743</v>
       </c>
-      <c r="B36" s="19" t="s">
-        <v>2614</v>
-      </c>
-      <c r="C36" s="20" t="s">
-        <v>205</v>
-      </c>
-      <c r="D36" s="19" t="s">
+      <c r="F36" s="16" t="s">
         <v>2744</v>
       </c>
-      <c r="E36" s="19" t="s">
+      <c r="G36" s="16" t="s">
         <v>2745</v>
       </c>
-      <c r="F36" s="19" t="s">
-        <v>2746</v>
-      </c>
-      <c r="G36" s="19" t="s">
-        <v>2747</v>
-      </c>
-      <c r="H36" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="I36" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="J36" s="19" t="s">
-        <v>79</v>
+      <c r="H36" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="I36" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="J36" s="16" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="37" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="18" t="s">
-        <v>2748</v>
+        <v>2746</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>2667</v>
+        <v>2614</v>
       </c>
       <c r="C37" s="20" t="s">
         <v>205</v>
       </c>
       <c r="D37" s="19" t="s">
+        <v>2747</v>
+      </c>
+      <c r="E37" s="19" t="s">
+        <v>2748</v>
+      </c>
+      <c r="F37" s="19" t="s">
         <v>2749</v>
       </c>
-      <c r="E37" s="19" t="s">
+      <c r="G37" s="19" t="s">
         <v>2750</v>
       </c>
-      <c r="F37" s="19" t="s">
+      <c r="H37" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="I37" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="J37" s="19" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="38" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" s="18" t="s">
         <v>2751</v>
       </c>
-      <c r="G37" s="19" t="s">
-        <v>2752</v>
-      </c>
-      <c r="H37" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="I37" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="J37" s="19" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="38" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A38" s="18" t="s">
-        <v>2753</v>
-      </c>
       <c r="B38" s="19" t="s">
-        <v>2729</v>
+        <v>146</v>
       </c>
       <c r="C38" s="20" t="s">
         <v>205</v>
       </c>
       <c r="D38" s="19" t="s">
+        <v>2752</v>
+      </c>
+      <c r="E38" s="19" t="s">
+        <v>2753</v>
+      </c>
+      <c r="F38" s="19" t="s">
         <v>2754</v>
       </c>
-      <c r="E38" s="19" t="s">
+      <c r="G38" s="19" t="s">
         <v>2755</v>
-      </c>
-      <c r="F38" s="19" t="s">
-        <v>2756</v>
-      </c>
-      <c r="G38" s="19" t="s">
-        <v>2757</v>
       </c>
       <c r="H38" s="19" t="s">
         <v>42</v>
@@ -14376,199 +14364,199 @@
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="18" t="s">
-        <v>2758</v>
+        <v>2756</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>2729</v>
+        <v>2728</v>
       </c>
       <c r="C39" s="20" t="s">
         <v>205</v>
       </c>
       <c r="D39" s="19" t="s">
+        <v>2757</v>
+      </c>
+      <c r="E39" s="19" t="s">
+        <v>2758</v>
+      </c>
+      <c r="F39" s="19" t="s">
         <v>2759</v>
       </c>
-      <c r="E39" s="19" t="s">
+      <c r="G39" s="19" t="s">
         <v>2760</v>
       </c>
-      <c r="F39" s="19" t="s">
+      <c r="H39" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="I39" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="J39" s="19" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="40" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" s="18" t="s">
         <v>2761</v>
       </c>
-      <c r="G39" s="19" t="s">
-        <v>2762</v>
-      </c>
-      <c r="H39" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="I39" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="J39" s="19" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="40" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A40" s="18" t="s">
-        <v>2763</v>
-      </c>
       <c r="B40" s="19" t="s">
-        <v>2729</v>
+        <v>2728</v>
       </c>
       <c r="C40" s="20" t="s">
         <v>205</v>
       </c>
       <c r="D40" s="19" t="s">
+        <v>2762</v>
+      </c>
+      <c r="E40" s="19" t="s">
+        <v>2763</v>
+      </c>
+      <c r="F40" s="19" t="s">
         <v>2764</v>
       </c>
-      <c r="E40" s="19" t="s">
+      <c r="G40" s="19" t="s">
         <v>2765</v>
       </c>
-      <c r="F40" s="19" t="s">
+      <c r="H40" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="I40" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="J40" s="19" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="41" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" s="18" t="s">
         <v>2766</v>
       </c>
-      <c r="G40" s="19" t="s">
+      <c r="B41" s="19" t="s">
+        <v>2728</v>
+      </c>
+      <c r="C41" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="D41" s="19" t="s">
         <v>2767</v>
       </c>
-      <c r="H40" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="I40" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="J40" s="19" t="s">
+      <c r="E41" s="19" t="s">
+        <v>2768</v>
+      </c>
+      <c r="F41" s="19" t="s">
+        <v>2769</v>
+      </c>
+      <c r="G41" s="19" t="s">
+        <v>2770</v>
+      </c>
+      <c r="H41" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="I41" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="J41" s="19" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="41" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="15" t="s">
-        <v>2768</v>
-      </c>
-      <c r="B41" s="16" t="s">
-        <v>2729</v>
-      </c>
-      <c r="C41" s="17" t="s">
+    <row r="42" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" s="15" t="s">
+        <v>2771</v>
+      </c>
+      <c r="B42" s="16" t="s">
+        <v>2728</v>
+      </c>
+      <c r="C42" s="17" t="s">
         <v>205</v>
       </c>
-      <c r="D41" s="16" t="s">
+      <c r="D42" s="16" t="s">
+        <v>2772</v>
+      </c>
+      <c r="E42" s="16" t="s">
+        <v>2773</v>
+      </c>
+      <c r="F42" s="16" t="s">
+        <v>2774</v>
+      </c>
+      <c r="G42" s="16" t="s">
+        <v>2775</v>
+      </c>
+      <c r="H42" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="I42" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="J42" s="16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" s="18" t="s">
+        <v>2776</v>
+      </c>
+      <c r="B43" s="19" t="s">
+        <v>2728</v>
+      </c>
+      <c r="C43" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="D43" s="19" t="s">
+        <v>2777</v>
+      </c>
+      <c r="E43" s="19" t="s">
+        <v>2778</v>
+      </c>
+      <c r="F43" s="19" t="s">
         <v>2769</v>
       </c>
-      <c r="E41" s="16" t="s">
-        <v>2770</v>
-      </c>
-      <c r="F41" s="16" t="s">
-        <v>2771</v>
-      </c>
-      <c r="G41" s="16" t="s">
-        <v>2772</v>
-      </c>
-      <c r="H41" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="I41" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="J41" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="42" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" s="18" t="s">
-        <v>2773</v>
-      </c>
-      <c r="B42" s="19" t="s">
-        <v>2729</v>
-      </c>
-      <c r="C42" s="20" t="s">
-        <v>205</v>
-      </c>
-      <c r="D42" s="19" t="s">
-        <v>2774</v>
-      </c>
-      <c r="E42" s="19" t="s">
-        <v>2775</v>
-      </c>
-      <c r="F42" s="19" t="s">
-        <v>2766</v>
-      </c>
-      <c r="G42" s="19" t="s">
-        <v>2776</v>
-      </c>
-      <c r="H42" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="I42" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="J42" s="19" t="s">
+      <c r="G43" s="19" t="s">
+        <v>2779</v>
+      </c>
+      <c r="H43" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="I43" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="J43" s="19" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="43" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43" s="11" t="s">
-        <v>2777</v>
-      </c>
-      <c r="B43" s="11"/>
-      <c r="C43" s="11"/>
-      <c r="D43" s="11"/>
-      <c r="E43" s="11"/>
-      <c r="F43" s="11"/>
-      <c r="G43" s="11"/>
-      <c r="H43" s="11"/>
-      <c r="I43" s="11"/>
-      <c r="J43" s="11"/>
-    </row>
-    <row r="44" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A44" s="15" t="s">
-        <v>2778</v>
-      </c>
-      <c r="B44" s="16" t="s">
-        <v>2667</v>
-      </c>
-      <c r="C44" s="17" t="s">
-        <v>701</v>
-      </c>
-      <c r="D44" s="16" t="s">
-        <v>2779</v>
-      </c>
-      <c r="E44" s="16" t="s">
+    <row r="44" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A44" s="11" t="s">
         <v>2780</v>
       </c>
-      <c r="F44" s="16" t="s">
-        <v>2781</v>
-      </c>
-      <c r="G44" s="16" t="s">
-        <v>2782</v>
-      </c>
-      <c r="H44" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="I44" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="J44" s="16" t="s">
-        <v>10</v>
-      </c>
+      <c r="B44" s="11"/>
+      <c r="C44" s="11"/>
+      <c r="D44" s="11"/>
+      <c r="E44" s="11"/>
+      <c r="F44" s="11"/>
+      <c r="G44" s="11"/>
+      <c r="H44" s="11"/>
+      <c r="I44" s="11"/>
+      <c r="J44" s="11"/>
     </row>
     <row r="45" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="15" t="s">
-        <v>2783</v>
+        <v>2781</v>
       </c>
       <c r="B45" s="16" t="s">
-        <v>2667</v>
+        <v>2646</v>
       </c>
       <c r="C45" s="17" t="s">
         <v>701</v>
       </c>
       <c r="D45" s="16" t="s">
+        <v>2782</v>
+      </c>
+      <c r="E45" s="16" t="s">
+        <v>2783</v>
+      </c>
+      <c r="F45" s="16" t="s">
         <v>2784</v>
       </c>
-      <c r="E45" s="16" t="s">
+      <c r="G45" s="16" t="s">
         <v>2785</v>
-      </c>
-      <c r="F45" s="16" t="s">
-        <v>2786</v>
-      </c>
-      <c r="G45" s="16" t="s">
-        <v>2787</v>
       </c>
       <c r="H45" s="16" t="s">
         <v>42</v>
@@ -14582,7 +14570,7 @@
     </row>
     <row r="46" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
-        <v>795</v>
+        <v>1070</v>
       </c>
       <c r="B46" s="11"/>
       <c r="C46" s="11"/>
@@ -14596,25 +14584,25 @@
     </row>
     <row r="47" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="18" t="s">
+        <v>2786</v>
+      </c>
+      <c r="B47" s="19" t="s">
+        <v>2651</v>
+      </c>
+      <c r="C47" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="D47" s="19" t="s">
+        <v>2787</v>
+      </c>
+      <c r="E47" s="19" t="s">
         <v>2788</v>
       </c>
-      <c r="B47" s="19" t="s">
+      <c r="F47" s="19" t="s">
         <v>2789</v>
       </c>
-      <c r="C47" s="20" t="s">
-        <v>224</v>
-      </c>
-      <c r="D47" s="19" t="s">
+      <c r="G47" s="19" t="s">
         <v>2790</v>
-      </c>
-      <c r="E47" s="19" t="s">
-        <v>2791</v>
-      </c>
-      <c r="F47" s="19" t="s">
-        <v>2792</v>
-      </c>
-      <c r="G47" s="19" t="s">
-        <v>2793</v>
       </c>
       <c r="H47" s="19" t="s">
         <v>42</v>
@@ -14626,27 +14614,27 @@
         <v>79</v>
       </c>
     </row>
-    <row r="48" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="18" t="s">
+        <v>2791</v>
+      </c>
+      <c r="B48" s="19" t="s">
+        <v>2651</v>
+      </c>
+      <c r="C48" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="D48" s="19" t="s">
+        <v>2792</v>
+      </c>
+      <c r="E48" s="19" t="s">
+        <v>2793</v>
+      </c>
+      <c r="F48" s="19" t="s">
         <v>2794</v>
       </c>
-      <c r="B48" s="19" t="s">
-        <v>2789</v>
-      </c>
-      <c r="C48" s="20" t="s">
-        <v>224</v>
-      </c>
-      <c r="D48" s="19" t="s">
+      <c r="G48" s="19" t="s">
         <v>2795</v>
-      </c>
-      <c r="E48" s="19" t="s">
-        <v>2796</v>
-      </c>
-      <c r="F48" s="19" t="s">
-        <v>2792</v>
-      </c>
-      <c r="G48" s="19" t="s">
-        <v>2797</v>
       </c>
       <c r="H48" s="19" t="s">
         <v>42</v>
@@ -14660,26 +14648,26 @@
     </row>
     <row r="49" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="18" t="s">
+        <v>2796</v>
+      </c>
+      <c r="B49" s="19" t="s">
+        <v>2651</v>
+      </c>
+      <c r="C49" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="D49" s="19" t="s">
+        <v>2797</v>
+      </c>
+      <c r="E49" s="19" t="s">
         <v>2798</v>
       </c>
-      <c r="B49" s="19" t="s">
-        <v>2789</v>
-      </c>
-      <c r="C49" s="20" t="s">
-        <v>224</v>
-      </c>
-      <c r="D49" s="19" t="s">
+      <c r="F49" s="19" t="s">
         <v>2799</v>
       </c>
-      <c r="E49" s="19" t="s">
+      <c r="G49" s="19" t="s">
         <v>2800</v>
       </c>
-      <c r="F49" s="19" t="s">
-        <v>2801</v>
-      </c>
-      <c r="G49" s="19" t="s">
-        <v>2802</v>
-      </c>
       <c r="H49" s="19" t="s">
         <v>42</v>
       </c>
@@ -14687,31 +14675,31 @@
         <v>42</v>
       </c>
       <c r="J49" s="19" t="s">
-        <v>79</v>
+        <v>328</v>
       </c>
     </row>
     <row r="50" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="18" t="s">
+        <v>2801</v>
+      </c>
+      <c r="B50" s="19" t="s">
+        <v>2651</v>
+      </c>
+      <c r="C50" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="D50" s="19" t="s">
+        <v>2802</v>
+      </c>
+      <c r="E50" s="19" t="s">
         <v>2803</v>
       </c>
-      <c r="B50" s="19" t="s">
+      <c r="F50" s="19" t="s">
         <v>2789</v>
       </c>
-      <c r="C50" s="20" t="s">
-        <v>224</v>
-      </c>
-      <c r="D50" s="19" t="s">
+      <c r="G50" s="19" t="s">
         <v>2804</v>
       </c>
-      <c r="E50" s="19" t="s">
-        <v>2805</v>
-      </c>
-      <c r="F50" s="19" t="s">
-        <v>2737</v>
-      </c>
-      <c r="G50" s="19" t="s">
-        <v>2806</v>
-      </c>
       <c r="H50" s="19" t="s">
         <v>42</v>
       </c>
@@ -14719,62 +14707,44 @@
         <v>42</v>
       </c>
       <c r="J50" s="19" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="51" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A51" s="18" t="s">
-        <v>2807</v>
-      </c>
-      <c r="B51" s="19" t="s">
-        <v>2789</v>
-      </c>
-      <c r="C51" s="20" t="s">
-        <v>224</v>
-      </c>
-      <c r="D51" s="19" t="s">
-        <v>2808</v>
-      </c>
-      <c r="E51" s="19" t="s">
-        <v>2809</v>
-      </c>
-      <c r="F51" s="19" t="s">
-        <v>2810</v>
-      </c>
-      <c r="G51" s="19" t="s">
-        <v>2811</v>
-      </c>
-      <c r="H51" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="I51" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="J51" s="19" t="s">
         <v>79</v>
       </c>
+    </row>
+    <row r="51" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A51" s="11" t="s">
+        <v>471</v>
+      </c>
+      <c r="B51" s="11"/>
+      <c r="C51" s="11"/>
+      <c r="D51" s="11"/>
+      <c r="E51" s="11"/>
+      <c r="F51" s="11"/>
+      <c r="G51" s="11"/>
+      <c r="H51" s="11"/>
+      <c r="I51" s="11"/>
+      <c r="J51" s="11"/>
     </row>
     <row r="52" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="18" t="s">
-        <v>2812</v>
+        <v>2805</v>
       </c>
       <c r="B52" s="19" t="s">
-        <v>2789</v>
+        <v>2651</v>
       </c>
       <c r="C52" s="20" t="s">
         <v>224</v>
       </c>
       <c r="D52" s="19" t="s">
-        <v>2813</v>
+        <v>2806</v>
       </c>
       <c r="E52" s="19" t="s">
-        <v>2814</v>
+        <v>2807</v>
       </c>
       <c r="F52" s="19" t="s">
-        <v>2815</v>
+        <v>2789</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>2816</v>
+        <v>2808</v>
       </c>
       <c r="H52" s="19" t="s">
         <v>42</v>
@@ -14783,30 +14753,30 @@
         <v>42</v>
       </c>
       <c r="J52" s="19" t="s">
-        <v>328</v>
+        <v>79</v>
       </c>
     </row>
     <row r="53" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="18" t="s">
-        <v>2817</v>
+        <v>2809</v>
       </c>
       <c r="B53" s="19" t="s">
-        <v>2789</v>
+        <v>2614</v>
       </c>
       <c r="C53" s="20" t="s">
         <v>224</v>
       </c>
       <c r="D53" s="19" t="s">
-        <v>2818</v>
+        <v>2810</v>
       </c>
       <c r="E53" s="19" t="s">
-        <v>2819</v>
+        <v>2811</v>
       </c>
       <c r="F53" s="19" t="s">
-        <v>2820</v>
+        <v>2812</v>
       </c>
       <c r="G53" s="19" t="s">
-        <v>2821</v>
+        <v>2813</v>
       </c>
       <c r="H53" s="19" t="s">
         <v>42</v>
@@ -14815,50 +14785,116 @@
         <v>42</v>
       </c>
       <c r="J53" s="19" t="s">
-        <v>328</v>
+        <v>79</v>
       </c>
     </row>
     <row r="54" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="18" t="s">
-        <v>2822</v>
+        <v>2814</v>
       </c>
       <c r="B54" s="19" t="s">
-        <v>2789</v>
+        <v>2646</v>
       </c>
       <c r="C54" s="20" t="s">
         <v>224</v>
       </c>
       <c r="D54" s="19" t="s">
+        <v>2815</v>
+      </c>
+      <c r="E54" s="19" t="s">
+        <v>2620</v>
+      </c>
+      <c r="F54" s="19" t="s">
+        <v>2816</v>
+      </c>
+      <c r="G54" s="19" t="s">
+        <v>2817</v>
+      </c>
+      <c r="H54" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="I54" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="J54" s="19" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="55" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" s="18" t="s">
+        <v>2818</v>
+      </c>
+      <c r="B55" s="19" t="s">
+        <v>2646</v>
+      </c>
+      <c r="C55" s="20" t="s">
+        <v>224</v>
+      </c>
+      <c r="D55" s="19" t="s">
+        <v>2819</v>
+      </c>
+      <c r="E55" s="19" t="s">
+        <v>2820</v>
+      </c>
+      <c r="F55" s="19" t="s">
+        <v>2821</v>
+      </c>
+      <c r="G55" s="19" t="s">
+        <v>2822</v>
+      </c>
+      <c r="H55" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="I55" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="J55" s="19" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="56" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A56" s="15" t="s">
         <v>2823</v>
       </c>
-      <c r="E54" s="19" t="s">
+      <c r="B56" s="16" t="s">
+        <v>2646</v>
+      </c>
+      <c r="C56" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="D56" s="16" t="s">
         <v>2824</v>
       </c>
-      <c r="F54" s="19" t="s">
-        <v>2792</v>
-      </c>
-      <c r="G54" s="19" t="s">
+      <c r="E56" s="16" t="s">
         <v>2825</v>
       </c>
-      <c r="H54" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="I54" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="J54" s="19" t="s">
-        <v>79</v>
+      <c r="F56" s="16" t="s">
+        <v>2826</v>
+      </c>
+      <c r="G56" s="16" t="s">
+        <v>2827</v>
+      </c>
+      <c r="H56" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="I56" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="J56" s="16" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A2:J2"/>
-  <mergeCells count="6">
+  <mergeCells count="8">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A21:J21"/>
+    <mergeCell ref="A29:J29"/>
     <mergeCell ref="A32:J32"/>
-    <mergeCell ref="A43:J43"/>
+    <mergeCell ref="A44:J44"/>
     <mergeCell ref="A46:J46"/>
+    <mergeCell ref="A51:J51"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>